<commit_message>
docs(okno-msk): validate Step 5A first execution
</commit_message>
<xml_diff>
--- a/extension/docs/kwork/KW001_AI_NATIVE_YANDEX_ALICE/tests/OKNO_MSK/STEP_05A_FIRST_EXECUTION_2026-09-08/STEP_05A_INFORMATION_GAIN_VALIDATION_REVIEW.xlsx
+++ b/extension/docs/kwork/KW001_AI_NATIVE_YANDEX_ALICE/tests/OKNO_MSK/STEP_05A_FIRST_EXECUTION_2026-09-08/STEP_05A_INFORMATION_GAIN_VALIDATION_REVIEW.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rb0d20677c6dd486c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funnel" sheetId="2" r:id="R20ff2cc8a37c428b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gates" sheetId="3" r:id="R100e7427590247e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="Rc4dfaca558dc44e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rf068f7d4b3ab4917"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funnel" sheetId="2" r:id="Ra02e409924de42b7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gates" sheetId="3" r:id="Rae7842b4144d47cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R2eeb3f884aa549ac"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -472,7 +472,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rad9f5b8e08f24a1f"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R13fc03e5ec074efc"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -502,7 +502,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R6857d8c091c04e8e"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R37080045055a46f1"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1022,7 +1022,7 @@
     <x:mergeCell ref="A13:F13"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R372ad7637235422a"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R245b7c9ac1054667"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
docs(okno-msk): record Step 5A validation readback
</commit_message>
<xml_diff>
--- a/extension/docs/kwork/KW001_AI_NATIVE_YANDEX_ALICE/tests/OKNO_MSK/STEP_05A_FIRST_EXECUTION_2026-09-08/STEP_05A_INFORMATION_GAIN_VALIDATION_REVIEW.xlsx
+++ b/extension/docs/kwork/KW001_AI_NATIVE_YANDEX_ALICE/tests/OKNO_MSK/STEP_05A_FIRST_EXECUTION_2026-09-08/STEP_05A_INFORMATION_GAIN_VALIDATION_REVIEW.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rf068f7d4b3ab4917"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funnel" sheetId="2" r:id="Ra02e409924de42b7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gates" sheetId="3" r:id="Rae7842b4144d47cc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R2eeb3f884aa549ac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rbdb8223cb8b540ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funnel" sheetId="2" r:id="R751a0a5b5e924ffa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gates" sheetId="3" r:id="Rd2eef9edef094c10"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R75e0c21982e143dc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -472,7 +472,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R13fc03e5ec074efc"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ra3d1e038e02f4267"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -502,7 +502,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R37080045055a46f1"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc6e76af64f23417c"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1022,7 +1022,7 @@
     <x:mergeCell ref="A13:F13"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R245b7c9ac1054667"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R68928ee991e24471"/>
 </x:worksheet>
 </file>
 

</xml_diff>

<commit_message>
docs(okno-msk): expand Step 5A client gap preview
</commit_message>
<xml_diff>
--- a/extension/docs/kwork/KW001_AI_NATIVE_YANDEX_ALICE/tests/OKNO_MSK/STEP_05A_FIRST_EXECUTION_2026-09-08/STEP_05A_INFORMATION_GAIN_VALIDATION_REVIEW.xlsx
+++ b/extension/docs/kwork/KW001_AI_NATIVE_YANDEX_ALICE/tests/OKNO_MSK/STEP_05A_FIRST_EXECUTION_2026-09-08/STEP_05A_INFORMATION_GAIN_VALIDATION_REVIEW.xlsx
@@ -2,10 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rbdb8223cb8b540ec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funnel" sheetId="2" r:id="R751a0a5b5e924ffa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gates" sheetId="3" r:id="Rd2eef9edef094c10"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="4" r:id="R75e0c21982e143dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Re20623532d5a4cd1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funnel" sheetId="2" r:id="Rc3e8a6ec074f48a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gates" sheetId="3" r:id="R56fc4e85b1514fa9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client Preview" sheetId="4" r:id="Rdb93804369b14966"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" r:id="R90561c46c6e94eaf"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -472,7 +473,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ra3d1e038e02f4267"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R960e2eaa019e4f46"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -502,7 +503,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rc6e76af64f23417c"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R628b76caae194cf2"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1022,7 +1023,7 @@
     <x:mergeCell ref="A13:F13"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R68928ee991e24471"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R11925708d316442a"/>
 </x:worksheet>
 </file>
 
@@ -2285,7 +2286,7 @@
     <x:col min="6" max="6" width="23.559999465942383" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="48" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="48" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="66.88999938964844" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="72.66999816894531" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="15" hidden="0" customHeight="1">
@@ -2592,7 +2593,7 @@
         <x:v>STEP_05A_CLIENT_FACING_COMPETITOR_GAP_PREVIEW_RU.md | STEP_05A_FIRST_EXECUTION_VALIDATION_QA.json</x:v>
       </x:c>
       <x:c r="E11" s="31" t="str">
-        <x:v>Plain-Russian preview contains 9 competitors, 44 pages, 7 confirmed directions, 2 unresolved directions, 16 prepared phrases and the no-new-page boundary</x:v>
+        <x:v>Plain-Russian preview contains all 16 accepted phrases in 7 directions; 7 exact-query checks; 11 visible query-domain cells; 12 ranking rows; explicit zero-selected-competitor case; 2 unresolved directions; no-new-page boundary</x:v>
       </x:c>
       <x:c r="F11" s="37" t="str">
         <x:v>OWNER_REVIEW_REQUIRED</x:v>
@@ -2604,7 +2605,7 @@
         <x:v>false</x:v>
       </x:c>
       <x:c r="I11" s="31" t="str">
-        <x:v>Read the preview and explicitly accept, request edits, or reject the client-facing presentation.</x:v>
+        <x:v>Read the revised preview and explicitly accept, request edits, or reject the client-facing presentation.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2613,6 +2614,499 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="42" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="48" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="42" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="42" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="42" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="14" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="15" hidden="0" customHeight="1">
+      <x:c r="A1" s="30" t="str">
+        <x:v>Клиентский обзор: найденные пропуски и проверенные позиции</x:v>
+      </x:c>
+      <x:c r="B1" s="30"/>
+      <x:c r="C1" s="30"/>
+      <x:c r="D1" s="30"/>
+      <x:c r="E1" s="30"/>
+      <x:c r="F1" s="30"/>
+      <x:c r="G1" s="31"/>
+      <x:c r="H1" s="31"/>
+    </x:row>
+    <x:row r="2" ht="15" hidden="0" customHeight="1">
+      <x:c r="A2" s="30"/>
+      <x:c r="B2" s="30"/>
+      <x:c r="C2" s="30"/>
+      <x:c r="D2" s="30"/>
+      <x:c r="E2" s="30"/>
+      <x:c r="F2" s="30"/>
+      <x:c r="G2" s="31"/>
+      <x:c r="H2" s="31"/>
+    </x:row>
+    <x:row r="3" ht="15" hidden="0" customHeight="1">
+      <x:c r="A3" s="31"/>
+      <x:c r="B3" s="31"/>
+      <x:c r="C3" s="31"/>
+      <x:c r="D3" s="31"/>
+      <x:c r="E3" s="31"/>
+      <x:c r="F3" s="31"/>
+      <x:c r="G3" s="31"/>
+      <x:c r="H3" s="31"/>
+    </x:row>
+    <x:row r="4" ht="15" hidden="0" customHeight="1">
+      <x:c r="A4" s="32" t="str">
+        <x:v>Этап отбора</x:v>
+      </x:c>
+      <x:c r="B4" s="33" t="str">
+        <x:v>Количество</x:v>
+      </x:c>
+      <x:c r="C4" s="31"/>
+      <x:c r="D4" s="32" t="str">
+        <x:v>Точный проверенный запрос</x:v>
+      </x:c>
+      <x:c r="E4" s="34" t="str">
+        <x:v>Найденные выбранные конкуренты</x:v>
+      </x:c>
+      <x:c r="F4" s="34" t="str">
+        <x:v>Точные позиции</x:v>
+      </x:c>
+      <x:c r="G4" s="34" t="str">
+        <x:v>Сайты</x:v>
+      </x:c>
+      <x:c r="H4" s="33" t="str">
+        <x:v>Позиции</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="15" hidden="0" customHeight="1">
+      <x:c r="A5" s="35" t="str">
+        <x:v>Самостоятельные направления</x:v>
+      </x:c>
+      <x:c r="B5" s="31" t="n">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="C5" s="31"/>
+      <x:c r="D5" s="31" t="str">
+        <x:v>гидроизоляция для открытого балкона</x:v>
+      </x:c>
+      <x:c r="E5" s="31" t="str">
+        <x:v>Выбранные конкуренты не найдены</x:v>
+      </x:c>
+      <x:c r="F5" s="31" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G5" s="31" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H5" s="31" t="n">
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="15" hidden="0" customHeight="1">
+      <x:c r="A6" s="35" t="str">
+        <x:v>Темы для Wordstat</x:v>
+      </x:c>
+      <x:c r="B6" s="31" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="C6" s="31"/>
+      <x:c r="D6" s="31" t="str">
+        <x:v>солнцезащитный стеклопакет</x:v>
+      </x:c>
+      <x:c r="E6" s="31" t="str">
+        <x:v>mosokna.ru; msk.okna-servise.com</x:v>
+      </x:c>
+      <x:c r="F6" s="31" t="str">
+        <x:v>mosokna.ru: 3; msk.okna-servise.com: 10</x:v>
+      </x:c>
+      <x:c r="G6" s="31" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H6" s="31" t="n">
+        <x:v>2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="15" hidden="0" customHeight="1">
+      <x:c r="A7" s="35" t="str">
+        <x:v>Возвращённые строки</x:v>
+      </x:c>
+      <x:c r="B7" s="31" t="n">
+        <x:v>160</x:v>
+      </x:c>
+      <x:c r="C7" s="31"/>
+      <x:c r="D7" s="31" t="str">
+        <x:v>многофункциональный стеклопакет что это</x:v>
+      </x:c>
+      <x:c r="E7" s="31" t="str">
+        <x:v>mosokna.ru; oknafactoria.ru; i-okna.ru</x:v>
+      </x:c>
+      <x:c r="F7" s="31" t="str">
+        <x:v>mosokna.ru: 2; oknafactoria.ru: 4; i-okna.ru: 5</x:v>
+      </x:c>
+      <x:c r="G7" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H7" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="15" hidden="0" customHeight="1">
+      <x:c r="A8" s="35" t="str">
+        <x:v>Кандидаты для проверки в Яндексе</x:v>
+      </x:c>
+      <x:c r="B8" s="31" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="C8" s="31"/>
+      <x:c r="D8" s="31" t="str">
+        <x:v>ударопрочный стеклопакет</x:v>
+      </x:c>
+      <x:c r="E8" s="31" t="str">
+        <x:v>oknafactoria.ru</x:v>
+      </x:c>
+      <x:c r="F8" s="31" t="str">
+        <x:v>oknafactoria.ru: 8</x:v>
+      </x:c>
+      <x:c r="G8" s="31" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H8" s="31" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="15" hidden="0" customHeight="1">
+      <x:c r="A9" s="35" t="str">
+        <x:v>Принятые фразы</x:v>
+      </x:c>
+      <x:c r="B9" s="31" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="C9" s="31"/>
+      <x:c r="D9" s="31" t="str">
+        <x:v>балконы под офис</x:v>
+      </x:c>
+      <x:c r="E9" s="31" t="str">
+        <x:v>fabrikaokon.ru</x:v>
+      </x:c>
+      <x:c r="F9" s="31" t="str">
+        <x:v>fabrikaokon.ru: 2</x:v>
+      </x:c>
+      <x:c r="G9" s="31" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H9" s="31" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="15" hidden="0" customHeight="1">
+      <x:c r="A10" s="31"/>
+      <x:c r="B10" s="31"/>
+      <x:c r="C10" s="31"/>
+      <x:c r="D10" s="31" t="str">
+        <x:v>шумоизоляция на крышу балкона</x:v>
+      </x:c>
+      <x:c r="E10" s="31" t="str">
+        <x:v>elit-balkon.ru</x:v>
+      </x:c>
+      <x:c r="F10" s="31" t="str">
+        <x:v>elit-balkon.ru: 9</x:v>
+      </x:c>
+      <x:c r="G10" s="31" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H10" s="31" t="n">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A11" s="32" t="str">
+        <x:v>Подтверждённое направление</x:v>
+      </x:c>
+      <x:c r="B11" s="33" t="str">
+        <x:v>Принятая поисковая фраза</x:v>
+      </x:c>
+      <x:c r="C11" s="31"/>
+      <x:c r="D11" s="31" t="str">
+        <x:v>армирование оконного профиля</x:v>
+      </x:c>
+      <x:c r="E11" s="31" t="str">
+        <x:v>fabrikaokon.ru; oknafactoria.ru; okna-germany.ru</x:v>
+      </x:c>
+      <x:c r="F11" s="31" t="str">
+        <x:v>fabrikaokon.ru: 1; oknafactoria.ru: 4, 7; okna-germany.ru: 8</x:v>
+      </x:c>
+      <x:c r="G11" s="31" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="H11" s="31" t="n">
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="15" hidden="0" customHeight="1">
+      <x:c r="A12" s="31" t="str">
+        <x:v>Гидроизоляция открытого балкона</x:v>
+      </x:c>
+      <x:c r="B12" s="31" t="str">
+        <x:v>гидроизоляция для открытого балкона</x:v>
+      </x:c>
+      <x:c r="C12" s="31"/>
+      <x:c r="D12" s="44" t="str">
+        <x:v>Итого</x:v>
+      </x:c>
+      <x:c r="E12" s="44" t="str">
+        <x:v>7 успешных проверок</x:v>
+      </x:c>
+      <x:c r="F12" s="44" t="str">
+        <x:v>11 сочетаний запрос + сайт / 12 строк выдачи</x:v>
+      </x:c>
+      <x:c r="G12" s="44" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="H12" s="44" t="n">
+        <x:v>12</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="15" hidden="0" customHeight="1">
+      <x:c r="A13" s="31" t="str">
+        <x:v>Гидроизоляция открытого балкона</x:v>
+      </x:c>
+      <x:c r="B13" s="31" t="str">
+        <x:v>гидроизоляция открытого балкона в частном доме</x:v>
+      </x:c>
+      <x:c r="C13" s="31"/>
+      <x:c r="D13" s="31"/>
+      <x:c r="E13" s="31"/>
+      <x:c r="F13" s="31"/>
+      <x:c r="G13" s="31"/>
+      <x:c r="H13" s="31"/>
+    </x:row>
+    <x:row r="14" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A14" s="31" t="str">
+        <x:v>Гидроизоляция открытого балкона</x:v>
+      </x:c>
+      <x:c r="B14" s="31" t="str">
+        <x:v>лучшая гидроизоляция для открытого балкона</x:v>
+      </x:c>
+      <x:c r="C14" s="31"/>
+      <x:c r="D14" s="37" t="str">
+        <x:v>По гидроизоляции открытого балкона: 0 выбранных конкурентов в первых десяти результатах; направление прошло по совокупности спроса, состава выдачи, бизнес-соответствия и новизны.</x:v>
+      </x:c>
+      <x:c r="E14" s="37"/>
+      <x:c r="F14" s="37"/>
+      <x:c r="G14" s="37"/>
+      <x:c r="H14" s="37"/>
+    </x:row>
+    <x:row r="15" ht="15" hidden="0" customHeight="1">
+      <x:c r="A15" s="31" t="str">
+        <x:v>Гидроизоляция открытого балкона</x:v>
+      </x:c>
+      <x:c r="B15" s="31" t="str">
+        <x:v>как сделать гидроизоляцию на открытом балконе</x:v>
+      </x:c>
+      <x:c r="C15" s="31"/>
+      <x:c r="D15" s="31"/>
+      <x:c r="E15" s="31"/>
+      <x:c r="F15" s="31"/>
+      <x:c r="G15" s="31"/>
+      <x:c r="H15" s="31"/>
+    </x:row>
+    <x:row r="16" ht="15" hidden="0" customHeight="1">
+      <x:c r="A16" s="31" t="str">
+        <x:v>Гидроизоляция открытого балкона</x:v>
+      </x:c>
+      <x:c r="B16" s="31" t="str">
+        <x:v>гидроизоляция открытого деревянного балкона</x:v>
+      </x:c>
+      <x:c r="C16" s="31"/>
+      <x:c r="D16" s="32" t="str">
+        <x:v>Нерешённые темы</x:v>
+      </x:c>
+      <x:c r="E16" s="33" t="str">
+        <x:v>Состояние</x:v>
+      </x:c>
+      <x:c r="F16" s="31"/>
+      <x:c r="G16" s="31"/>
+      <x:c r="H16" s="31"/>
+    </x:row>
+    <x:row r="17" ht="15" hidden="0" customHeight="1">
+      <x:c r="A17" s="31" t="str">
+        <x:v>Гидроизоляция открытого балкона</x:v>
+      </x:c>
+      <x:c r="B17" s="31" t="str">
+        <x:v>гидроизоляция балконной плиты открытого балкона</x:v>
+      </x:c>
+      <x:c r="C17" s="31"/>
+      <x:c r="D17" s="31" t="str">
+        <x:v>окна для старого фонда</x:v>
+      </x:c>
+      <x:c r="E17" s="31" t="str">
+        <x:v>Оставлена до будущей проверки</x:v>
+      </x:c>
+      <x:c r="F17" s="31"/>
+      <x:c r="G17" s="31"/>
+      <x:c r="H17" s="31"/>
+    </x:row>
+    <x:row r="18" ht="15" hidden="0" customHeight="1">
+      <x:c r="A18" s="31" t="str">
+        <x:v>Солнцезащитные стеклопакеты</x:v>
+      </x:c>
+      <x:c r="B18" s="31" t="str">
+        <x:v>солнцезащитный стеклопакет</x:v>
+      </x:c>
+      <x:c r="C18" s="31"/>
+      <x:c r="D18" s="31" t="str">
+        <x:v>кладовая на балконе</x:v>
+      </x:c>
+      <x:c r="E18" s="31" t="str">
+        <x:v>Оставлена до будущей проверки</x:v>
+      </x:c>
+      <x:c r="F18" s="31"/>
+      <x:c r="G18" s="31"/>
+      <x:c r="H18" s="31"/>
+    </x:row>
+    <x:row r="19" ht="15" hidden="0" customHeight="1">
+      <x:c r="A19" s="31" t="str">
+        <x:v>Солнцезащитные стеклопакеты</x:v>
+      </x:c>
+      <x:c r="B19" s="31" t="str">
+        <x:v>солнцезащитное стекло в стеклопакете</x:v>
+      </x:c>
+      <x:c r="C19" s="31"/>
+      <x:c r="D19" s="31"/>
+      <x:c r="E19" s="31"/>
+      <x:c r="F19" s="31"/>
+      <x:c r="G19" s="31"/>
+      <x:c r="H19" s="31"/>
+    </x:row>
+    <x:row r="20" ht="15" hidden="0" customHeight="1">
+      <x:c r="A20" s="31" t="str">
+        <x:v>Солнцезащитные стеклопакеты</x:v>
+      </x:c>
+      <x:c r="B20" s="31" t="str">
+        <x:v>солнцезащитный стеклопакет rehau</x:v>
+      </x:c>
+      <x:c r="C20" s="31"/>
+      <x:c r="D20" s="37" t="str">
+        <x:v>16 фраз не означают автоматическое создание новых страниц: до реального релиза требуется обычная дальнейшая обработка.</x:v>
+      </x:c>
+      <x:c r="E20" s="37"/>
+      <x:c r="F20" s="37"/>
+      <x:c r="G20" s="37"/>
+      <x:c r="H20" s="37"/>
+    </x:row>
+    <x:row r="21" ht="15" hidden="0" customHeight="1">
+      <x:c r="A21" s="31" t="str">
+        <x:v>Особенности многофункциональных стеклопакетов</x:v>
+      </x:c>
+      <x:c r="B21" s="31" t="str">
+        <x:v>многофункциональный стеклопакет что это</x:v>
+      </x:c>
+      <x:c r="C21" s="31"/>
+      <x:c r="D21" s="31"/>
+      <x:c r="E21" s="31"/>
+      <x:c r="F21" s="31"/>
+      <x:c r="G21" s="31"/>
+      <x:c r="H21" s="31"/>
+    </x:row>
+    <x:row r="22" ht="15" hidden="0" customHeight="1">
+      <x:c r="A22" s="31" t="str">
+        <x:v>Ударопрочные стеклопакеты</x:v>
+      </x:c>
+      <x:c r="B22" s="31" t="str">
+        <x:v>ударопрочный стеклопакет</x:v>
+      </x:c>
+      <x:c r="C22" s="31"/>
+      <x:c r="D22" s="31"/>
+      <x:c r="E22" s="31"/>
+      <x:c r="F22" s="31"/>
+      <x:c r="G22" s="31"/>
+      <x:c r="H22" s="31"/>
+    </x:row>
+    <x:row r="23" ht="15" hidden="0" customHeight="1">
+      <x:c r="A23" s="31" t="str">
+        <x:v>Переоборудование балкона под рабочее место</x:v>
+      </x:c>
+      <x:c r="B23" s="31" t="str">
+        <x:v>балконы под офис</x:v>
+      </x:c>
+      <x:c r="C23" s="31"/>
+      <x:c r="D23" s="31"/>
+      <x:c r="E23" s="31"/>
+      <x:c r="F23" s="31"/>
+      <x:c r="G23" s="31"/>
+      <x:c r="H23" s="31"/>
+    </x:row>
+    <x:row r="24" ht="15" hidden="0" customHeight="1">
+      <x:c r="A24" s="31" t="str">
+        <x:v>Шумоизоляция крыши балкона</x:v>
+      </x:c>
+      <x:c r="B24" s="31" t="str">
+        <x:v>шумоизоляция на крышу балкона</x:v>
+      </x:c>
+      <x:c r="C24" s="31"/>
+      <x:c r="D24" s="31"/>
+      <x:c r="E24" s="31"/>
+      <x:c r="F24" s="31"/>
+      <x:c r="G24" s="31"/>
+      <x:c r="H24" s="31"/>
+    </x:row>
+    <x:row r="25" ht="15" hidden="0" customHeight="1">
+      <x:c r="A25" s="31" t="str">
+        <x:v>Шумоизоляция крыши балкона</x:v>
+      </x:c>
+      <x:c r="B25" s="31" t="str">
+        <x:v>шумоизоляция крыши балкона от дождя</x:v>
+      </x:c>
+      <x:c r="C25" s="31"/>
+      <x:c r="D25" s="31"/>
+      <x:c r="E25" s="31"/>
+      <x:c r="F25" s="31"/>
+      <x:c r="G25" s="31"/>
+      <x:c r="H25" s="31"/>
+    </x:row>
+    <x:row r="26" ht="15" hidden="0" customHeight="1">
+      <x:c r="A26" s="31" t="str">
+        <x:v>Шумоизоляция крыши балкона</x:v>
+      </x:c>
+      <x:c r="B26" s="31" t="str">
+        <x:v>шумоизоляция крыши балкона изнутри от дождя</x:v>
+      </x:c>
+      <x:c r="C26" s="31"/>
+      <x:c r="D26" s="31"/>
+      <x:c r="E26" s="31"/>
+      <x:c r="F26" s="31"/>
+      <x:c r="G26" s="31"/>
+      <x:c r="H26" s="31"/>
+    </x:row>
+    <x:row r="27" ht="15" hidden="0" customHeight="1">
+      <x:c r="A27" s="31" t="str">
+        <x:v>Армирование оконного профиля</x:v>
+      </x:c>
+      <x:c r="B27" s="31" t="str">
+        <x:v>армирование оконного профиля</x:v>
+      </x:c>
+      <x:c r="C27" s="31"/>
+      <x:c r="D27" s="31"/>
+      <x:c r="E27" s="31"/>
+      <x:c r="F27" s="31"/>
+      <x:c r="G27" s="31"/>
+      <x:c r="H27" s="31"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:F2"/>
+    <x:mergeCell ref="D14:H14"/>
+    <x:mergeCell ref="D20:H20"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>

</xml_diff>